<commit_message>
Update attendees for quiz: quize-v2 — fevin@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/quize-v2/attendees.xlsx
+++ b/quizzes/quize-v2/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -455,9 +455,50 @@
         <v>Grade</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>fevin@gmail.com</v>
+      </c>
+      <c r="B2" t="str">
+        <v>as</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Quize V2</v>
+      </c>
+      <c r="D2" t="str">
+        <v>8/13/2026, 12:04:23 AM</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="M2" t="str">
+        <v>F</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: quize-v2 — sample@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/quize-v2/attendees.xlsx
+++ b/quizzes/quize-v2/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -496,9 +496,50 @@
         <v>F</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>sample@gmail.com</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Fejin FM</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Quize V2</v>
+      </c>
+      <c r="D3" t="str">
+        <v>8/13/2026, 12:07:41 AM</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3" t="str">
+        <v>50.00</v>
+      </c>
+      <c r="M3" t="str">
+        <v>D</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: quize-v2 — admin@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/quize-v2/attendees.xlsx
+++ b/quizzes/quize-v2/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>Quize V2</v>
       </c>
       <c r="D2" t="str">
-        <v>8/13/2026, 12:04:23 AM</v>
+        <v>13/8/2026, 12:04:23 am</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -507,7 +507,7 @@
         <v>Quize V2</v>
       </c>
       <c r="D3" t="str">
-        <v>8/13/2026, 12:07:41 AM</v>
+        <v>13/8/2026, 12:07:41 am</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -534,12 +534,53 @@
         <v>50.00</v>
       </c>
       <c r="M3" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>admin@gmail.com</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Quize V2</v>
+      </c>
+      <c r="D4" t="str">
+        <v>13/8/2026, 11:15:46 am</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4" t="str">
+        <v>50.00</v>
+      </c>
+      <c r="M4" t="str">
         <v>D</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: quize-v2 — fejinf@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/quize-v2/attendees.xlsx
+++ b/quizzes/quize-v2/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>Quize V2</v>
       </c>
       <c r="D2" t="str">
-        <v>13/8/2026, 12:04:23 am</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -507,7 +507,7 @@
         <v>Quize V2</v>
       </c>
       <c r="D3" t="str">
-        <v>13/8/2026, 12:07:41 am</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -548,7 +548,7 @@
         <v>Quize V2</v>
       </c>
       <c r="D4" t="str">
-        <v>13/8/2026, 11:15:46 am</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -575,12 +575,53 @@
         <v>50.00</v>
       </c>
       <c r="M4" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>fejinf@clarium.tech</v>
+      </c>
+      <c r="B5" t="str">
+        <v>as</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Quize V2</v>
+      </c>
+      <c r="D5" t="str">
+        <v>13/8/2026, 12:03:19 pm</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5" t="str">
+        <v>50.00</v>
+      </c>
+      <c r="M5" t="str">
         <v>D</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>